<commit_message>
add change for set resid daryaft code
</commit_message>
<xml_diff>
--- a/cache/resid_sepidar_template.xlsx
+++ b/cache/resid_sepidar_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milad\Desktop\milad_repo\cache\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dorsa-Co\Desktop\temp\pichNew\cache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BCF9634-0FBD-41C3-A680-628780B34891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E97E17-9106-40E3-A3F3-862D8EAD2AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{83EEF9FF-486E-45B8-B529-E2369E6CE5FE}"/>
   </bookViews>
@@ -28,9 +28,6 @@
     <t>رسيد دريافت نوع دريافت</t>
   </si>
   <si>
-    <t>رسيد دريافت طرف مقابل</t>
-  </si>
-  <si>
     <t>رسيد دريافت شماره</t>
   </si>
   <si>
@@ -137,6 +134,9 @@
   </si>
   <si>
     <t>رسيد دريافت استقراري</t>
+  </si>
+  <si>
+    <t>رسيد دريافت کد</t>
   </si>
 </sst>
 </file>
@@ -555,115 +555,115 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:39" x14ac:dyDescent="0.2">

</xml_diff>